<commit_message>
Sync the seed exercise xlsx with its csv, and add zip+pictures import for the library
The seed exercise .xlsx had drifted from the .csv - the nine gym-equipment
exercises added in an earlier round never made it into the .xlsx, so the
Excel template only ever seeded 38 of 47 real exercises. Fixed by extracting
the missing rows straight from the .csv (the source of truth) rather than
retyping them, verified against the app's own xlsx parser.

Also gives the Exercise Library its own "spreadsheet + pictures (.zip)"
import, mirroring the plan importer's existing one exactly - down to reusing
its readPlanZipBundle()/PlanZipBundle unchanged, since that function was
already generic and never actually plan-specific. Fixes a stale claim in
TemplatesScreen that said this path didn't exist for the library.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed-data/strongman_exercise_database.xlsx
+++ b/seed-data/strongman_exercise_database.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="461" uniqueCount="314">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="370">
   <si>
     <t xml:space="preserve">Exercise ID</t>
   </si>
@@ -965,6 +965,174 @@
     <t xml:space="preserve">If you already have a list of exercises written down somewhere (a document, notes app, an old spreadsheet, or a coach's program), you can ask an AI assistant to fill in this template for you instead of doing it by hand. Attach this file to your AI assistant of choice and adapt this prompt:
 "I'm attaching a spreadsheet template for a workout-tracking app's exercise library. Fill in the 'Exercises' tab using the exercise list I describe below, following the 'Legend' tab's column definitions exactly - Difficulty must be exactly one of Beginner/Intermediate/Advanced. Leave the 'Embedding' column blank unless I specifically tell you a video should be embedded, and never invent a video link yourself. Don't guess or invent values for any column I haven't given you information for - leave those cells blank instead. Return the completed spreadsheet in the same column order as the template.
 [describe your exercises here, or paste your existing list]"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EX039</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable Row (Seated)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable Machine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Squeeze the shoulder blades together at the finish; keep a slight lean back throughout, not a big rock.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avoid rounding the lower back to add range at the finish - stop the pull where your torso naturally stops moving.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.youtube.com/results?search_query=Seated+Cable+Row+form+technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EX040</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable Tricep Pushdown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Arms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep elbows pinned to your sides throughout; let the triceps do the work rather than leaning on the bar with body weight.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Don't let the elbows drift forward as the weight gets heavy - that shifts load onto the shoulders.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.youtube.com/results?search_query=Cable+Tricep+Pushdown+form+technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EX041</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leg Press</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leg Press Machine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A safer entry point than a free-bar squat for building leg strength - feet shoulder-width on the platform; lower until knees reach roughly 90 degrees.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Never let the lower back round off the pad at the bottom of the rep; don't lock the knees out hard at the top.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.youtube.com/results?search_query=Leg+Press+form+technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EX042</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lat Pulldown</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lat Pulldown Machine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pull the bar to the upper chest, driving the elbows down and back rather than pulling with the arms alone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avoid leaning back excessively or using momentum to move the weight.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.youtube.com/results?search_query=Lat+Pulldown+form+technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EX043</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smith Machine Squat</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Smith Machine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The fixed bar path makes this a good option for practicing squat depth and tempo without needing a spotter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Position feet slightly forward of the bar, not directly under it, to keep the movement path comfortable for the knees.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.youtube.com/results?search_query=Smith+Machine+Squat+form+technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EX044</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leg Extension</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Legs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leg Extension Machine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An isolation move for the quads; extend the knees fully then lower under control rather than dropping the weight stack.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avoid using momentum by swinging into the first few reps - start each set under control.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.youtube.com/results?search_query=Leg+Extension+Machine+form+technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EX045</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seated Leg Curl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leg Curl Machine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An isolation move for the hamstrings; curl through a full range and pause briefly at full contraction.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keep the hips pressed into the seat throughout - don't let them lift to help move the weight.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.youtube.com/results?search_query=Seated+Leg+Curl+form+technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EX046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chest Press Machine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A guided alternative to the bench press for building pressing strength without needing a spotter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Adjust the seat height first so the handles line up with mid-chest, not the shoulders or the collarbone.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.youtube.com/results?search_query=Chest+Press+Machine+form+technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EX047</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wrist Wrench Roll</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wrist Wrench</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A lever (often a bar or PVC pipe with a rope and weight attached) rotated by the wrists to roll the weight up, then lowered under control; builds forearm and wrist strength for grip-heavy lifts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Start light - this is a small-muscle-group movement and forearms fatigue and strain easily if the load jumps too fast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.youtube.com/results?search_query=Wrist+Roller+forearm+training+technique</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Picture</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional filename of a photo for this exercise, e.g. 'lat_pulldown.jpg'. Only works when importing via 'From spreadsheet + pictures (.zip)' - zip this spreadsheet together with the image files it names (using exactly these filenames; folder structure inside the zip doesn't matter) and import that zip instead of the plain spreadsheet. The photo attaches to the resulting exercise. Leave blank for rows that don't need one.</t>
   </si>
 </sst>
 </file>
@@ -1411,7 +1579,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L39"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -1426,6 +1594,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="24"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1465,6 +1634,9 @@
       <c r="L1" s="1" t="s">
         <v>310</v>
       </c>
+      <c r="M1" s="1" t="s">
+        <v>368</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
@@ -2794,6 +2966,321 @@
       </c>
       <c r="K39" s="5" t="s">
         <v>293</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="2" t="s">
+        <v>314</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>315</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>234</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>317</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="B41" s="4" t="s">
+        <v>321</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H41" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="J41" s="4" t="s">
+        <v>324</v>
+      </c>
+      <c r="K41" s="4" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>327</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>218</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>328</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>329</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>330</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="B43" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="D43" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="E43" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>334</v>
+      </c>
+      <c r="G43" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I43" s="4" t="s">
+        <v>335</v>
+      </c>
+      <c r="J43" s="4" t="s">
+        <v>336</v>
+      </c>
+      <c r="K43" s="4" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="s">
+        <v>338</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>339</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>340</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>341</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>342</v>
+      </c>
+      <c r="K44" s="2" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>344</v>
+      </c>
+      <c r="B45" s="4" t="s">
+        <v>345</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="D45" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E45" s="4" t="s">
+        <v>346</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>347</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>348</v>
+      </c>
+      <c r="J45" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="K45" s="4" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="2" t="s">
+        <v>351</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>233</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>346</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>353</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>354</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="K46" s="2" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="J47" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="K47" s="4" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="2" t="s">
+        <v>362</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>363</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>364</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>365</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>366</v>
+      </c>
+      <c r="K48" s="2" t="s">
+        <v>367</v>
       </c>
     </row>
   </sheetData>
@@ -2830,7 +3317,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B20"/>
+  <dimension ref="A1:B21"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -2970,6 +3457,14 @@
         <v>313</v>
       </c>
       <c r="B20" s="7"/>
+    </row>
+    <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="9" t="s">
+        <v>368</v>
+      </c>
+      <c r="B21" s="10" t="s">
+        <v>369</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Fix five trainer-report gaps found by actually reading a generated PDF
Header now names the trainer (Plans.createdBy), both spreadsheet
templates gained authorship columns (Created By / Author), trainees can
attach a per-set note for the trainer (LoggedSets.notes), the full log
is rebuilt as one pw.Table so a workout can no longer split mid-exercise
with its border left open, and lib/logic/rx_deviation.dart flags fewer
sets, under-target reps/weight, near-failure RPE, and trainee notes as
colored tags instead of requiring a line-by-line read to spot a
difference from the prescription.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/seed-data/strongman_exercise_database.xlsx
+++ b/seed-data/strongman_exercise_database.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="563" uniqueCount="370">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="565" uniqueCount="372">
   <si>
     <t xml:space="preserve">Exercise ID</t>
   </si>
@@ -963,7 +963,7 @@
   </si>
   <si>
     <t xml:space="preserve">If you already have a list of exercises written down somewhere (a document, notes app, an old spreadsheet, or a coach's program), you can ask an AI assistant to fill in this template for you instead of doing it by hand. Attach this file to your AI assistant of choice and adapt this prompt:
-"I'm attaching a spreadsheet template for a workout-tracking app's exercise library. Fill in the 'Exercises' tab using the exercise list I describe below, following the 'Legend' tab's column definitions exactly - Difficulty must be exactly one of Beginner/Intermediate/Advanced. Leave the 'Embedding' column blank unless I specifically tell you a video should be embedded, and never invent a video link yourself. Don't guess or invent values for any column I haven't given you information for - leave those cells blank instead. Return the completed spreadsheet in the same column order as the template.
+"I'm attaching a spreadsheet template for a workout-tracking app's exercise library. Fill in the 'Exercises' tab using the exercise list I describe below, following the 'Legend' tab's column definitions exactly - Difficulty must be exactly one of Beginner/Intermediate/Advanced. Leave the 'Embedding' column blank unless I specifically tell you a video should be embedded, and never invent a video link yourself. Fill in 'Author' only if I tell you this list is from a specific coach/creator, with their name exactly as I give it to you. Don't guess or invent values for any column I haven't given you information for - leave those cells blank instead. Return the completed spreadsheet in the same column order as the template.
 [describe your exercises here, or paste your existing list]"</t>
   </si>
   <si>
@@ -1133,6 +1133,12 @@
   </si>
   <si>
     <t xml:space="preserve">Optional filename of a photo for this exercise, e.g. 'lat_pulldown.jpg'. Only works when importing via 'From spreadsheet + pictures (.zip)' - zip this spreadsheet together with the image files it names (using exactly these filenames; folder structure inside the zip doesn't matter) and import that zip instead of the plain spreadsheet. The photo attaches to the resulting exercise. Leave blank for rows that don't need one.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Author</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional free-text creator name for this exercise (e.g. a coach's name). Every exercise sharing one Author value shows up as a single named, manageable group in the Exercise Library's own "Manage libraries &amp; blocks" screen - export, rename, or delete that whole imported set at once. Leave blank for an exercise you're not attributing to anyone in particular.</t>
   </si>
 </sst>
 </file>
@@ -1579,7 +1585,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M48"/>
+  <dimension ref="A1:N48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -1595,6 +1601,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="20"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1636,6 +1643,9 @@
       </c>
       <c r="M1" s="1" t="s">
         <v>368</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>370</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3317,7 +3327,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
@@ -3464,6 +3474,14 @@
       </c>
       <c r="B21" s="10" t="s">
         <v>369</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
+        <v>370</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>